<commit_message>
Update products - 28/09/2026 14:51:02.78
</commit_message>
<xml_diff>
--- a/Description Converter.xlsx
+++ b/Description Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\chatloot-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1330F9D-C747-4EC1-8524-04A46272EB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6409F5-DE52-49FA-BF0E-D158AA6C1D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2580" yWindow="2220" windowWidth="35820" windowHeight="18660" xr2:uid="{F2BFF4DE-C334-4DE3-8C39-32DBA17BB15B}"/>
   </bookViews>
@@ -39,27 +39,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>✨ Custom Spotify Music Widget for Twitch ✨</t>
-  </si>
-  <si>
-    <t>Bring your stream to life with a fully customizable Spotify widget designed to showcase your current music 💜</t>
-  </si>
-  <si>
-    <t>Features:</t>
-  </si>
-  <si>
-    <t>★ Display your currently playing Spotify track directly on your stream 🎵</t>
-  </si>
-  <si>
-    <t>★ Fully customize the text, colors, fonts, layout, icons and overall appearance to match your stream aesthetic 🎨</t>
-  </si>
-  <si>
-    <t>★ Compatible with OBS, Streamlabs, and other streaming software that supports browser sources 🖥️</t>
-  </si>
-  <si>
-    <t>★ Easy-to-follow setup instructions are included so you can get your widget up and running quickly 🙌</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>🎃 Trick or Treat 3D Halloween Widget! 👻</t>
+  </si>
+  <si>
+    <t>★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬</t>
+  </si>
+  <si>
+    <t>★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃</t>
+  </si>
+  <si>
+    <t>★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡</t>
+  </si>
+  <si>
+    <t>★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️</t>
+  </si>
+  <si>
+    <t>★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨</t>
+  </si>
+  <si>
+    <t>★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️</t>
+  </si>
+  <si>
+    <t>★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆</t>
+  </si>
+  <si>
+    <t>★ Multilingual Friendly: All text can be edited into any language 🌐</t>
+  </si>
+  <si>
+    <t>★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡</t>
   </si>
 </sst>
 </file>
@@ -443,7 +452,7 @@
       </c>
       <c r="C1" t="str">
         <f>SUBSTITUTE(IF(A1&lt;&gt;"",A1&amp;"\n\n",""),"?","")</f>
-        <v>✨ Custom Spotify Music Widget for Twitch ✨\n\n</v>
+        <v>🎃 Trick or Treat 3D Halloween Widget! 👻\n\n</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -458,67 +467,79 @@
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C32" si="0">SUBSTITUTE(IF(A3&lt;&gt;"",A3&amp;"\n",""),"?","")</f>
-        <v>Bring your stream to life with a fully customizable Spotify widget designed to showcase your current music 💜\n</v>
+        <v>★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬\n</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃\n</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>Features:\n</v>
+        <v>★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡\n</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️\n</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>★ Display your currently playing Spotify track directly on your stream 🎵\n</v>
+        <v>★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨\n</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️\n</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>★ Fully customize the text, colors, fonts, layout, icons and overall appearance to match your stream aesthetic 🎨\n</v>
+        <v>★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆\n</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>★ Multilingual Friendly: All text can be edited into any language 🌐\n</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>★ Compatible with OBS, Streamlabs, and other streaming software that supports browser sources 🖥️\n</v>
+        <v>★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡\n</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -528,12 +549,9 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>6</v>
-      </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
-        <v>★ Easy-to-follow setup instructions are included so you can get your widget up and running quickly 🙌\n</v>
+        <v/>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -653,13 +671,13 @@
     <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f>_xlfn.CONCAT(C1:C33)</f>
-        <v>✨ Custom Spotify Music Widget for Twitch ✨\n\nBring your stream to life with a fully customizable Spotify widget designed to showcase your current music 💜\nFeatures:\n★ Display your currently playing Spotify track directly on your stream 🎵\n★ Fully customize the text, colors, fonts, layout, icons and overall appearance to match your stream aesthetic 🎨\n★ Compatible with OBS, Streamlabs, and other streaming software that supports browser sources 🖥️\n★ Easy-to-follow setup instructions are included so you can get your widget up and running quickly 🙌\n</v>
+        <v>🎃 Trick or Treat 3D Halloween Widget! 👻\n\n★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬\n★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃\n★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡\n★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️\n★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨\n★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️\n★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆\n★ Multilingual Friendly: All text can be edited into any language 🌐\n★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡\n</v>
       </c>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
         <f>"""description"""&amp;": "&amp;""""&amp;C34&amp;""""&amp;","</f>
-        <v>"description": "✨ Custom Spotify Music Widget for Twitch ✨\n\nBring your stream to life with a fully customizable Spotify widget designed to showcase your current music 💜\nFeatures:\n★ Display your currently playing Spotify track directly on your stream 🎵\n★ Fully customize the text, colors, fonts, layout, icons and overall appearance to match your stream aesthetic 🎨\n★ Compatible with OBS, Streamlabs, and other streaming software that supports browser sources 🖥️\n★ Easy-to-follow setup instructions are included so you can get your widget up and running quickly 🙌\n",</v>
+        <v>"description": "🎃 Trick or Treat 3D Halloween Widget! 👻\n\n★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬\n★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃\n★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡\n★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️\n★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨\n★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️\n★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆\n★ Multilingual Friendly: All text can be edited into any language 🌐\n★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡\n",</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update products - 29/09/2026 11:18:27.62
</commit_message>
<xml_diff>
--- a/Description Converter.xlsx
+++ b/Description Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\chatloot-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6409F5-DE52-49FA-BF0E-D158AA6C1D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73ED584-DFCD-4D78-8440-D3E2D1D73081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2580" yWindow="2220" windowWidth="35820" windowHeight="18660" xr2:uid="{F2BFF4DE-C334-4DE3-8C39-32DBA17BB15B}"/>
   </bookViews>
@@ -39,36 +39,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>🎃 Trick or Treat 3D Halloween Widget! 👻</t>
+    <t>Bat Stream Decoration 🦇</t>
   </si>
   <si>
-    <t>★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬</t>
+    <t>★ Options: Includes animated and static versions</t>
   </si>
   <si>
-    <t>★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃</t>
+    <t>★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software</t>
   </si>
   <si>
-    <t>★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡</t>
-  </si>
-  <si>
-    <t>★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️</t>
-  </si>
-  <si>
-    <t>★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨</t>
-  </si>
-  <si>
-    <t>★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️</t>
-  </si>
-  <si>
-    <t>★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆</t>
-  </si>
-  <si>
-    <t>★ Multilingual Friendly: All text can be edited into any language 🌐</t>
-  </si>
-  <si>
-    <t>★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡</t>
+    <t>★ Compatibility: Works with Twitch, Kick and Youtube</t>
   </si>
 </sst>
 </file>
@@ -452,7 +434,7 @@
       </c>
       <c r="C1" t="str">
         <f>SUBSTITUTE(IF(A1&lt;&gt;"",A1&amp;"\n\n",""),"?","")</f>
-        <v>🎃 Trick or Treat 3D Halloween Widget! 👻\n\n</v>
+        <v>Bat Stream Decoration 🦇\n\n</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -467,79 +449,61 @@
       </c>
       <c r="C3" t="str">
         <f t="shared" ref="C3:C32" si="0">SUBSTITUTE(IF(A3&lt;&gt;"",A3&amp;"\n",""),"?","")</f>
-        <v>★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬\n</v>
+        <v>★ Options: Includes animated and static versions\n</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
-        <v>★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃\n</v>
+        <v/>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡\n</v>
+        <v>★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software\n</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️\n</v>
+        <v/>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨\n</v>
+        <v>★ Compatibility: Works with Twitch, Kick and Youtube\n</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️\n</v>
+        <v/>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆\n</v>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v>★ Multilingual Friendly: All text can be edited into any language 🌐\n</v>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡\n</v>
+        <v/>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -671,13 +635,13 @@
     <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f>_xlfn.CONCAT(C1:C33)</f>
-        <v>🎃 Trick or Treat 3D Halloween Widget! 👻\n\n★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬\n★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃\n★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡\n★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️\n★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨\n★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️\n★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆\n★ Multilingual Friendly: All text can be edited into any language 🌐\n★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡\n</v>
+        <v>Bat Stream Decoration 🦇\n\n★ Options: Includes animated and static versions\n★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software\n★ Compatibility: Works with Twitch, Kick and Youtube\n</v>
       </c>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
         <f>"""description"""&amp;": "&amp;""""&amp;C34&amp;""""&amp;","</f>
-        <v>"description": "🎃 Trick or Treat 3D Halloween Widget! 👻\n\n★ 3D Halloween Scene: Viewers lootboxes open inside a cozy Halloween bedroom filled with spooky decorations🕯️🍬\n★ Chat Command: Viewers can type !tot (or any custom word you choose) to unlock and collect unique tricks or treats 🎃\n★ Channel Points Ready: Perfect as a channel point reward to boost chat engagement 🧡\n★ Never Repeats: No duplicate tricks or treats in a row – every surprise feels fresh ✔️\n★ Personalized Shoutouts: The viewer’s username pops up inside the 3D scene for a magical interactive touch ✨\n★ Customizable Everything: Change fonts, colors, and scene lighting to match your Halloween stream theme 🕷️\n★ Collect &amp; Compete: Viewers can check their collection and climb the leaderboard for most treats collected 🏆\n★ Multilingual Friendly: All text can be edited into any language 🌐\n★ Easy Setup: Simple one-click install through StreamElements – works with OBS, Streamlabs, and any browser source ⚡\n",</v>
+        <v>"description": "Bat Stream Decoration 🦇\n\n★ Options: Includes animated and static versions\n★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software\n★ Compatibility: Works with Twitch, Kick and Youtube\n",</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update products - 29/09/2026 11:29:04.38
</commit_message>
<xml_diff>
--- a/Description Converter.xlsx
+++ b/Description Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\chatloot-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73ED584-DFCD-4D78-8440-D3E2D1D73081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678003A4-EBA8-4CED-9885-5DB6EA215BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2580" yWindow="2220" windowWidth="35820" windowHeight="18660" xr2:uid="{F2BFF4DE-C334-4DE3-8C39-32DBA17BB15B}"/>
   </bookViews>
@@ -39,18 +39,78 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Bat Stream Decoration 🦇</t>
-  </si>
-  <si>
-    <t>★ Options: Includes animated and static versions</t>
-  </si>
-  <si>
-    <t>★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software</t>
-  </si>
-  <si>
-    <t>★ Compatibility: Works with Twitch, Kick and Youtube</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+  <si>
+    <t>🎀✨ Kawaii Christmas Streamer Bundle ✨🎀</t>
+  </si>
+  <si>
+    <t>Make your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖</t>
+  </si>
+  <si>
+    <t>🎁 What’s inside:</t>
+  </si>
+  <si>
+    <t>✨ Kawaii Christmas Overlays (4 Layouts)</t>
+  </si>
+  <si>
+    <t>Christmas overlays in multiple layouts so you can choose the perfect look for your stream.</t>
+  </si>
+  <si>
+    <t>💬 Chat Widget</t>
+  </si>
+  <si>
+    <t>A cute chat widget that keeps messages clear while adding festive charm.</t>
+  </si>
+  <si>
+    <t>⏳ Countdown Widget</t>
+  </si>
+  <si>
+    <t>Christmas countdown timer</t>
+  </si>
+  <si>
+    <t>❄️ Snow Widget</t>
+  </si>
+  <si>
+    <t>Soft falling pastel snow animation to give your stream magical cozy vibes.</t>
+  </si>
+  <si>
+    <t>🎄 Fairy Lights</t>
+  </si>
+  <si>
+    <t>Cute pastel decorations hanging across your screen to add extra holiday sweetness.</t>
+  </si>
+  <si>
+    <t>🎁 Penguin Lootbox</t>
+  </si>
+  <si>
+    <t>Let viewers open a lootbox full of cute surprises.</t>
+  </si>
+  <si>
+    <t>💗 Sub Badges</t>
+  </si>
+  <si>
+    <t>Festive themed badges to brighten up your chat.</t>
+  </si>
+  <si>
+    <t>🎀 Twitch Panels</t>
+  </si>
+  <si>
+    <t>Matching Christmas panels for a perfectly cohesive look.</t>
+  </si>
+  <si>
+    <t>🎅 Advent Calendar Widget</t>
+  </si>
+  <si>
+    <t>Reveal a surprise each day of December.</t>
+  </si>
+  <si>
+    <t>❄️ Mystery Drink Widget</t>
+  </si>
+  <si>
+    <t>Viewers can redeem a festive hot chocolate.</t>
+  </si>
+  <si>
+    <t>Easy plug-and-play browser-source widgets for OBS / Streamlabs!</t>
   </si>
 </sst>
 </file>
@@ -434,7 +494,7 @@
       </c>
       <c r="C1" t="str">
         <f>SUBSTITUTE(IF(A1&lt;&gt;"",A1&amp;"\n\n",""),"?","")</f>
-        <v>Bat Stream Decoration 🦇\n\n</v>
+        <v>🎀✨ Kawaii Christmas Streamer Bundle ✨🎀\n\n</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -448,200 +508,260 @@
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C32" si="0">SUBSTITUTE(IF(A3&lt;&gt;"",A3&amp;"\n",""),"?","")</f>
-        <v>★ Options: Includes animated and static versions\n</v>
+        <f t="shared" ref="C3:C31" si="0">SUBSTITUTE(IF(A3&lt;&gt;"",A3&amp;"\n",""),"?","")</f>
+        <v>Make your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖\n</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>🎁 What’s inside:\n</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software\n</v>
+        <v>✨ Kawaii Christmas Overlays (4 Layouts)\n</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Christmas overlays in multiple layouts so you can choose the perfect look for your stream.\n</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>★ Compatibility: Works with Twitch, Kick and Youtube\n</v>
+        <v>💬 Chat Widget\n</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
+        <v>A cute chat widget that keeps messages clear while adding festive charm.\n</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="0"/>
+        <v>⏳ Countdown Widget\n</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
+        <v>Christmas countdown timer\n</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="0"/>
+        <v>❄️ Snow Widget\n</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="0"/>
+        <v>Soft falling pastel snow animation to give your stream magical cozy vibes.\n</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="str">
+        <f t="shared" si="0"/>
+        <v>🎄 Fairy Lights\n</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="0"/>
+        <v>Cute pastel decorations hanging across your screen to add extra holiday sweetness.\n</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="0"/>
+        <v>🎁 Penguin Lootbox\n</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="0"/>
+        <v>Let viewers open a lootbox full of cute surprises.\n</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="0"/>
+        <v>💗 Sub Badges\n</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="0"/>
+        <v>Festive themed badges to brighten up your chat.\n</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="0"/>
+        <v>🎀 Twitch Panels\n</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="0"/>
+        <v>Matching Christmas panels for a perfectly cohesive look.\n</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="0"/>
+        <v>🎅 Advent Calendar Widget\n</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="0"/>
+        <v>Reveal a surprise each day of December.\n</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="0"/>
+        <v>❄️ Mystery Drink Widget\n</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="0"/>
+        <v>Viewers can redeem a festive hot chocolate.\n</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="0"/>
+        <v>Easy plug-and-play browser-source widgets for OBS / Streamlabs!\n</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C26" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C9" t="str">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C27" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C10" t="str">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C28" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C11" t="str">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C29" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C12" t="str">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C30" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C13" t="str">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C31" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C14" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C18" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C20" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C21" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C22" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C23" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C24" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C26" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C27" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C28" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C30" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C31" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C32" t="str">
-        <f t="shared" si="0"/>
+        <f>SUBSTITUTE(IF(A29&lt;&gt;"",A29&amp;"\n",""),"?","")</f>
         <v/>
       </c>
     </row>
     <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f>_xlfn.CONCAT(C1:C33)</f>
-        <v>Bat Stream Decoration 🦇\n\n★ Options: Includes animated and static versions\n★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software\n★ Compatibility: Works with Twitch, Kick and Youtube\n</v>
+        <v>🎀✨ Kawaii Christmas Streamer Bundle ✨🎀\n\nMake your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖\n🎁 What’s inside:\n✨ Kawaii Christmas Overlays (4 Layouts)\nChristmas overlays in multiple layouts so you can choose the perfect look for your stream.\n💬 Chat Widget\nA cute chat widget that keeps messages clear while adding festive charm.\n⏳ Countdown Widget\nChristmas countdown timer\n❄️ Snow Widget\nSoft falling pastel snow animation to give your stream magical cozy vibes.\n🎄 Fairy Lights\nCute pastel decorations hanging across your screen to add extra holiday sweetness.\n🎁 Penguin Lootbox\nLet viewers open a lootbox full of cute surprises.\n💗 Sub Badges\nFestive themed badges to brighten up your chat.\n🎀 Twitch Panels\nMatching Christmas panels for a perfectly cohesive look.\n🎅 Advent Calendar Widget\nReveal a surprise each day of December.\n❄️ Mystery Drink Widget\nViewers can redeem a festive hot chocolate.\nEasy plug-and-play browser-source widgets for OBS / Streamlabs!\n</v>
       </c>
     </row>
     <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
-        <f>"""description"""&amp;": "&amp;""""&amp;C34&amp;""""&amp;","</f>
-        <v>"description": "Bat Stream Decoration 🦇\n\n★ Options: Includes animated and static versions\n★ Quick Set-Up: Load into OBS, Streamlabs or your preferred streaming software\n★ Compatibility: Works with Twitch, Kick and Youtube\n",</v>
+        <f>"    "&amp;"""description"""&amp;": "&amp;""""&amp;C34&amp;""""&amp;","</f>
+        <v xml:space="preserve">    "description": "🎀✨ Kawaii Christmas Streamer Bundle ✨🎀\n\nMake your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖\n🎁 What’s inside:\n✨ Kawaii Christmas Overlays (4 Layouts)\nChristmas overlays in multiple layouts so you can choose the perfect look for your stream.\n💬 Chat Widget\nA cute chat widget that keeps messages clear while adding festive charm.\n⏳ Countdown Widget\nChristmas countdown timer\n❄️ Snow Widget\nSoft falling pastel snow animation to give your stream magical cozy vibes.\n🎄 Fairy Lights\nCute pastel decorations hanging across your screen to add extra holiday sweetness.\n🎁 Penguin Lootbox\nLet viewers open a lootbox full of cute surprises.\n💗 Sub Badges\nFestive themed badges to brighten up your chat.\n🎀 Twitch Panels\nMatching Christmas panels for a perfectly cohesive look.\n🎅 Advent Calendar Widget\nReveal a surprise each day of December.\n❄️ Mystery Drink Widget\nViewers can redeem a festive hot chocolate.\nEasy plug-and-play browser-source widgets for OBS / Streamlabs!\n",</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update products - 29/09/2026 12:09:58.08
</commit_message>
<xml_diff>
--- a/Description Converter.xlsx
+++ b/Description Converter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\chatloot-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678003A4-EBA8-4CED-9885-5DB6EA215BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F33A70E-0690-4E54-A40B-ECFBBF44E240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2580" yWindow="2220" windowWidth="35820" windowHeight="18660" xr2:uid="{F2BFF4DE-C334-4DE3-8C39-32DBA17BB15B}"/>
   </bookViews>
@@ -39,78 +39,102 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>🎀✨ Kawaii Christmas Streamer Bundle ✨🎀</t>
-  </si>
-  <si>
-    <t>Make your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖</t>
-  </si>
-  <si>
-    <t>🎁 What’s inside:</t>
-  </si>
-  <si>
-    <t>✨ Kawaii Christmas Overlays (4 Layouts)</t>
-  </si>
-  <si>
-    <t>Christmas overlays in multiple layouts so you can choose the perfect look for your stream.</t>
-  </si>
-  <si>
-    <t>💬 Chat Widget</t>
-  </si>
-  <si>
-    <t>A cute chat widget that keeps messages clear while adding festive charm.</t>
-  </si>
-  <si>
-    <t>⏳ Countdown Widget</t>
-  </si>
-  <si>
-    <t>Christmas countdown timer</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>❄️ Snow Widget</t>
   </si>
   <si>
-    <t>Soft falling pastel snow animation to give your stream magical cozy vibes.</t>
-  </si>
-  <si>
-    <t>🎄 Fairy Lights</t>
-  </si>
-  <si>
-    <t>Cute pastel decorations hanging across your screen to add extra holiday sweetness.</t>
-  </si>
-  <si>
-    <t>🎁 Penguin Lootbox</t>
-  </si>
-  <si>
-    <t>Let viewers open a lootbox full of cute surprises.</t>
-  </si>
-  <si>
-    <t>💗 Sub Badges</t>
-  </si>
-  <si>
-    <t>Festive themed badges to brighten up your chat.</t>
-  </si>
-  <si>
-    <t>🎀 Twitch Panels</t>
-  </si>
-  <si>
-    <t>Matching Christmas panels for a perfectly cohesive look.</t>
-  </si>
-  <si>
     <t>🎅 Advent Calendar Widget</t>
   </si>
   <si>
-    <t>Reveal a surprise each day of December.</t>
-  </si>
-  <si>
-    <t>❄️ Mystery Drink Widget</t>
-  </si>
-  <si>
-    <t>Viewers can redeem a festive hot chocolate.</t>
-  </si>
-  <si>
-    <t>Easy plug-and-play browser-source widgets for OBS / Streamlabs!</t>
+    <t>🎄✨ Ultimate Christmas Twitch Stream Bundle ✨🎄</t>
+  </si>
+  <si>
+    <t>This all-in-one holiday bundle includes everything you need to decorate, engage your viewers, and add magical Christmas vibes to your channel 🌟</t>
+  </si>
+  <si>
+    <t>What’s Included:</t>
+  </si>
+  <si>
+    <t>✨ Christmas Stream Overlay</t>
+  </si>
+  <si>
+    <t>• Comes with 4 layout options</t>
+  </si>
+  <si>
+    <t>🎁 Lootbox Widget</t>
+  </si>
+  <si>
+    <t>• Christmas gnome lootbox</t>
+  </si>
+  <si>
+    <t>• Great for channel points or chat commands</t>
+  </si>
+  <si>
+    <t>✨ Christmas Fairy String Lights</t>
+  </si>
+  <si>
+    <t>• Festive fairy lights</t>
+  </si>
+  <si>
+    <t>• Place anywhere on your stream</t>
+  </si>
+  <si>
+    <t>⭐ Christmas Sub Badges (23 styles)</t>
+  </si>
+  <si>
+    <t>• High-quality PNGs</t>
+  </si>
+  <si>
+    <t>• Cute, festive designs for all your subscriber tiers</t>
+  </si>
+  <si>
+    <t>💬 Christmas Twitch Panels</t>
+  </si>
+  <si>
+    <t>• Matching festive designs</t>
+  </si>
+  <si>
+    <t>• Multiple colour options included</t>
+  </si>
+  <si>
+    <t>• Interactive daily reveal for December</t>
+  </si>
+  <si>
+    <t>• Perfect for viewer engagement</t>
+  </si>
+  <si>
+    <t>💬 Christmas Chat Widget</t>
+  </si>
+  <si>
+    <t>• Themed chat overlay</t>
+  </si>
+  <si>
+    <t>• Matches the rest of the bundle</t>
+  </si>
+  <si>
+    <t>☕ Mystery Drink Widget</t>
+  </si>
+  <si>
+    <t>• Username + random festive drink reveal</t>
+  </si>
+  <si>
+    <t>• Collectible system &amp; commands available</t>
+  </si>
+  <si>
+    <t>• Gentle animated snowfall overlay</t>
+  </si>
+  <si>
+    <t>• Works on any scene</t>
+  </si>
+  <si>
+    <t>⏰ Christmas Countdown Widget</t>
+  </si>
+  <si>
+    <t>• Live countdown to Christmas Day</t>
+  </si>
+  <si>
+    <t>• Customizable colours + fonts</t>
   </si>
 </sst>
 </file>
@@ -490,11 +514,11 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C1" t="str">
         <f>SUBSTITUTE(IF(A1&lt;&gt;"",A1&amp;"\n\n",""),"?","")</f>
-        <v>🎀✨ Kawaii Christmas Streamer Bundle ✨🎀\n\n</v>
+        <v>🎄✨ Ultimate Christmas Twitch Stream Bundle ✨🎄\n\n</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -505,263 +529,289 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C31" si="0">SUBSTITUTE(IF(A3&lt;&gt;"",A3&amp;"\n",""),"?","")</f>
-        <v>Make your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖\n</v>
+        <f t="shared" ref="C3:C32" si="0">SUBSTITUTE(IF(A3&lt;&gt;"",A3&amp;"\n",""),"?","")</f>
+        <v>This all-in-one holiday bundle includes everything you need to decorate, engage your viewers, and add magical Christmas vibes to your channel 🌟\n</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
-        <v>🎁 What’s inside:\n</v>
+        <v>What’s Included:\n</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>✨ Kawaii Christmas Overlays (4 Layouts)\n</v>
+        <v>✨ Christmas Stream Overlay\n</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>Christmas overlays in multiple layouts so you can choose the perfect look for your stream.\n</v>
+        <v>• Comes with 4 layout options\n</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>💬 Chat Widget\n</v>
+        <v>🎁 Lootbox Widget\n</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>A cute chat widget that keeps messages clear while adding festive charm.\n</v>
+        <v>• Christmas gnome lootbox\n</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>⏳ Countdown Widget\n</v>
+        <v>• Great for channel points or chat commands\n</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v>Christmas countdown timer\n</v>
+        <v>✨ Christmas Fairy String Lights\n</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>❄️ Snow Widget\n</v>
+        <v>• Festive fairy lights\n</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="0"/>
-        <v>Soft falling pastel snow animation to give your stream magical cozy vibes.\n</v>
+        <v>• Place anywhere on your stream\n</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
-        <v>🎄 Fairy Lights\n</v>
+        <v>⭐ Christmas Sub Badges (23 styles)\n</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
-        <v>Cute pastel decorations hanging across your screen to add extra holiday sweetness.\n</v>
+        <v>• High-quality PNGs\n</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
-        <v>🎁 Penguin Lootbox\n</v>
+        <v>• Cute, festive designs for all your subscriber tiers\n</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C16" t="str">
         <f t="shared" si="0"/>
-        <v>Let viewers open a lootbox full of cute surprises.\n</v>
+        <v>💬 Christmas Twitch Panels\n</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="0"/>
-        <v>💗 Sub Badges\n</v>
+        <v>• Matching festive designs\n</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="0"/>
-        <v>Festive themed badges to brighten up your chat.\n</v>
+        <v>• Multiple colour options included\n</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
-        <v>🎀 Twitch Panels\n</v>
+        <v>🎅 Advent Calendar Widget\n</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
-        <v>Matching Christmas panels for a perfectly cohesive look.\n</v>
+        <v>• Interactive daily reveal for December\n</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
-        <v>🎅 Advent Calendar Widget\n</v>
+        <v>• Perfect for viewer engagement\n</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
-        <v>Reveal a surprise each day of December.\n</v>
+        <v>💬 Christmas Chat Widget\n</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="0"/>
-        <v>❄️ Mystery Drink Widget\n</v>
+        <v>• Themed chat overlay\n</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="0"/>
-        <v>Viewers can redeem a festive hot chocolate.\n</v>
+        <v>• Matches the rest of the bundle\n</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="0"/>
-        <v>Easy plug-and-play browser-source widgets for OBS / Streamlabs!\n</v>
+        <v>☕ Mystery Drink Widget\n</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
       <c r="C26" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>• Username + random festive drink reveal\n</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
       <c r="C27" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>• Collectible system &amp; commands available\n</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>0</v>
+      </c>
       <c r="C28" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>❄️ Snow Widget\n</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>• Gentle animated snowfall overlay\n</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>28</v>
+      </c>
       <c r="C30" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>• Works on any scene\n</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
       <c r="C31" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>⏰ Christmas Countdown Widget\n</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
       <c r="C32" t="str">
-        <f>SUBSTITUTE(IF(A29&lt;&gt;"",A29&amp;"\n",""),"?","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+        <f t="shared" si="0"/>
+        <v>• Live countdown to Christmas Day\n</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f>_xlfn.CONCAT(C1:C33)</f>
-        <v>🎀✨ Kawaii Christmas Streamer Bundle ✨🎀\n\nMake your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖\n🎁 What’s inside:\n✨ Kawaii Christmas Overlays (4 Layouts)\nChristmas overlays in multiple layouts so you can choose the perfect look for your stream.\n💬 Chat Widget\nA cute chat widget that keeps messages clear while adding festive charm.\n⏳ Countdown Widget\nChristmas countdown timer\n❄️ Snow Widget\nSoft falling pastel snow animation to give your stream magical cozy vibes.\n🎄 Fairy Lights\nCute pastel decorations hanging across your screen to add extra holiday sweetness.\n🎁 Penguin Lootbox\nLet viewers open a lootbox full of cute surprises.\n💗 Sub Badges\nFestive themed badges to brighten up your chat.\n🎀 Twitch Panels\nMatching Christmas panels for a perfectly cohesive look.\n🎅 Advent Calendar Widget\nReveal a surprise each day of December.\n❄️ Mystery Drink Widget\nViewers can redeem a festive hot chocolate.\nEasy plug-and-play browser-source widgets for OBS / Streamlabs!\n</v>
-      </c>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+        <v>🎄✨ Ultimate Christmas Twitch Stream Bundle ✨🎄\n\nThis all-in-one holiday bundle includes everything you need to decorate, engage your viewers, and add magical Christmas vibes to your channel 🌟\nWhat’s Included:\n✨ Christmas Stream Overlay\n• Comes with 4 layout options\n🎁 Lootbox Widget\n• Christmas gnome lootbox\n• Great for channel points or chat commands\n✨ Christmas Fairy String Lights\n• Festive fairy lights\n• Place anywhere on your stream\n⭐ Christmas Sub Badges (23 styles)\n• High-quality PNGs\n• Cute, festive designs for all your subscriber tiers\n💬 Christmas Twitch Panels\n• Matching festive designs\n• Multiple colour options included\n🎅 Advent Calendar Widget\n• Interactive daily reveal for December\n• Perfect for viewer engagement\n💬 Christmas Chat Widget\n• Themed chat overlay\n• Matches the rest of the bundle\n☕ Mystery Drink Widget\n• Username + random festive drink reveal\n• Collectible system &amp; commands available\n❄️ Snow Widget\n• Gentle animated snowfall overlay\n• Works on any scene\n⏰ Christmas Countdown Widget\n• Live countdown to Christmas Day\n</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
         <f>"    "&amp;"""description"""&amp;": "&amp;""""&amp;C34&amp;""""&amp;","</f>
-        <v xml:space="preserve">    "description": "🎀✨ Kawaii Christmas Streamer Bundle ✨🎀\n\nMake your holiday streams extra cute, cozy, and magical! This all-in-one Christmas bundle wraps your entire setup in adorable holiday charm so your viewers feel like they’ve stepped into a sweet winter wonderland. ❄️💖\n🎁 What’s inside:\n✨ Kawaii Christmas Overlays (4 Layouts)\nChristmas overlays in multiple layouts so you can choose the perfect look for your stream.\n💬 Chat Widget\nA cute chat widget that keeps messages clear while adding festive charm.\n⏳ Countdown Widget\nChristmas countdown timer\n❄️ Snow Widget\nSoft falling pastel snow animation to give your stream magical cozy vibes.\n🎄 Fairy Lights\nCute pastel decorations hanging across your screen to add extra holiday sweetness.\n🎁 Penguin Lootbox\nLet viewers open a lootbox full of cute surprises.\n💗 Sub Badges\nFestive themed badges to brighten up your chat.\n🎀 Twitch Panels\nMatching Christmas panels for a perfectly cohesive look.\n🎅 Advent Calendar Widget\nReveal a surprise each day of December.\n❄️ Mystery Drink Widget\nViewers can redeem a festive hot chocolate.\nEasy plug-and-play browser-source widgets for OBS / Streamlabs!\n",</v>
+        <v xml:space="preserve">    "description": "🎄✨ Ultimate Christmas Twitch Stream Bundle ✨🎄\n\nThis all-in-one holiday bundle includes everything you need to decorate, engage your viewers, and add magical Christmas vibes to your channel 🌟\nWhat’s Included:\n✨ Christmas Stream Overlay\n• Comes with 4 layout options\n🎁 Lootbox Widget\n• Christmas gnome lootbox\n• Great for channel points or chat commands\n✨ Christmas Fairy String Lights\n• Festive fairy lights\n• Place anywhere on your stream\n⭐ Christmas Sub Badges (23 styles)\n• High-quality PNGs\n• Cute, festive designs for all your subscriber tiers\n💬 Christmas Twitch Panels\n• Matching festive designs\n• Multiple colour options included\n🎅 Advent Calendar Widget\n• Interactive daily reveal for December\n• Perfect for viewer engagement\n💬 Christmas Chat Widget\n• Themed chat overlay\n• Matches the rest of the bundle\n☕ Mystery Drink Widget\n• Username + random festive drink reveal\n• Collectible system &amp; commands available\n❄️ Snow Widget\n• Gentle animated snowfall overlay\n• Works on any scene\n⏰ Christmas Countdown Widget\n• Live countdown to Christmas Day\n",</v>
       </c>
     </row>
   </sheetData>

</xml_diff>